<commit_message>
Added for IO Expander. Vivado added shared control of display qspi for ioX. Vitis added code for IOX 1 - next add for IOX 2
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAF132C-004D-4610-8E4D-8641E1E96A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24600B9E-6803-400C-98DA-93218E386613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="206">
   <si>
     <t>G13</t>
   </si>
@@ -612,6 +612,48 @@
   </si>
   <si>
     <t>Signal Select 1=BNC, 0=Oscillator (gpio2_io_o_0[7])</t>
+  </si>
+  <si>
+    <t>IOX_SCLK</t>
+  </si>
+  <si>
+    <t>IOX_MOSI</t>
+  </si>
+  <si>
+    <t>IO Expander common SPI SCLK</t>
+  </si>
+  <si>
+    <t>IO Expandeer common SPI MOSI</t>
+  </si>
+  <si>
+    <t>IOX_RESET</t>
+  </si>
+  <si>
+    <t>IO Expander common Reset (active low)</t>
+  </si>
+  <si>
+    <t>UI_CSn[1]</t>
+  </si>
+  <si>
+    <t>IO Expander 1 chip select (active low)</t>
+  </si>
+  <si>
+    <t>UI_CSn[2]</t>
+  </si>
+  <si>
+    <t>IO Expander 2 chip select (active low)</t>
+  </si>
+  <si>
+    <t>IOX_MISO</t>
+  </si>
+  <si>
+    <t>IO Expander common SPI MISO</t>
+  </si>
+  <si>
+    <t>IOX_2_IRQ</t>
+  </si>
+  <si>
+    <t>IO Expander 2 Interrupt</t>
   </si>
 </sst>
 </file>
@@ -696,12 +738,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1045,19 +1087,19 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>133</v>
       </c>
       <c r="H4" t="s">
@@ -1065,13 +1107,13 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
       <c r="H5" s="3" t="s">
         <v>160</v>
       </c>
@@ -1188,7 +1230,7 @@
       <c r="C12" t="s">
         <v>95</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>185</v>
       </c>
       <c r="E12" t="s">
@@ -1205,7 +1247,7 @@
       <c r="C13" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="5" t="s">
         <v>171</v>
       </c>
       <c r="E13" t="s">
@@ -1222,7 +1264,7 @@
       <c r="C14" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>172</v>
       </c>
       <c r="E14" t="s">
@@ -1239,7 +1281,7 @@
       <c r="C15" t="s">
         <v>98</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>173</v>
       </c>
       <c r="E15" t="s">
@@ -1269,13 +1311,13 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1452,13 +1494,13 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -1470,6 +1512,12 @@
       <c r="C32" t="s">
         <v>75</v>
       </c>
+      <c r="D32" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E32" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
@@ -1481,6 +1529,12 @@
       <c r="C33" t="s">
         <v>76</v>
       </c>
+      <c r="D33" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E33" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -1492,6 +1546,12 @@
       <c r="C34" t="s">
         <v>77</v>
       </c>
+      <c r="D34" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="E34" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -1503,6 +1563,12 @@
       <c r="C35" t="s">
         <v>78</v>
       </c>
+      <c r="D35" t="s">
+        <v>196</v>
+      </c>
+      <c r="E35" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
@@ -1547,6 +1613,12 @@
       <c r="C39" t="s">
         <v>80</v>
       </c>
+      <c r="D39" t="s">
+        <v>204</v>
+      </c>
+      <c r="E39" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -1558,6 +1630,12 @@
       <c r="C40" t="s">
         <v>81</v>
       </c>
+      <c r="D40" t="s">
+        <v>200</v>
+      </c>
+      <c r="E40" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -1569,6 +1647,12 @@
       <c r="C41" t="s">
         <v>82</v>
       </c>
+      <c r="D41" t="s">
+        <v>198</v>
+      </c>
+      <c r="E41" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
@@ -1593,13 +1677,13 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -1735,10 +1819,10 @@
       <c r="C53" t="s">
         <v>73</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D53" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E53" s="7" t="s">
+      <c r="E53" s="6" t="s">
         <v>187</v>
       </c>
     </row>
@@ -1782,13 +1866,13 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Added second IO expander and clean up of how the main test loop works - everything known to be working
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24600B9E-6803-400C-98DA-93218E386613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1702360-672E-400F-B1F2-7E9E79B50DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="220">
   <si>
     <t>G13</t>
   </si>
@@ -602,12 +602,6 @@
     <t>TEST_IO_0</t>
   </si>
   <si>
-    <t>Timer 1 Test Signal (gpio2_io_o_0[1] = TIMER_2_OUTPUT)</t>
-  </si>
-  <si>
-    <t>Timer 2 Test Signal (gpio2_io_o_0[0] =  TIMER_1_OUTPUT)</t>
-  </si>
-  <si>
     <t>Audio Enable = 1, Disable = 0 (gpio2_io_o_0[6])</t>
   </si>
   <si>
@@ -623,9 +617,6 @@
     <t>IO Expander common SPI SCLK</t>
   </si>
   <si>
-    <t>IO Expandeer common SPI MOSI</t>
-  </si>
-  <si>
     <t>IOX_RESET</t>
   </si>
   <si>
@@ -654,6 +645,57 @@
   </si>
   <si>
     <t>IO Expander 2 Interrupt</t>
+  </si>
+  <si>
+    <t>IO Expander common SPI MOSI</t>
+  </si>
+  <si>
+    <t>Timer 1 Test Signal (gpio2_io_o_0[0] =  TIMER_1_OUTPUT)</t>
+  </si>
+  <si>
+    <t>Timer 2 Test Signal (gpio2_io_o_0[1] = TIMER_2_OUTPUT)</t>
+  </si>
+  <si>
+    <t>J4.13</t>
+  </si>
+  <si>
+    <t>J4.15</t>
+  </si>
+  <si>
+    <t>CK_IO2</t>
+  </si>
+  <si>
+    <t>P14</t>
+  </si>
+  <si>
+    <t>TEST_IRQ</t>
+  </si>
+  <si>
+    <t>T11</t>
+  </si>
+  <si>
+    <t>CK_IO3</t>
+  </si>
+  <si>
+    <t>CK_IO4</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>ADC_IRQ_DONE</t>
+  </si>
+  <si>
+    <t>T14</t>
+  </si>
+  <si>
+    <t>CK_IO5</t>
+  </si>
+  <si>
+    <t>DISPLAY_CSn - not used - display uses JD1 - J4.1 for CSn</t>
+  </si>
+  <si>
+    <t>MB_RESET</t>
   </si>
 </sst>
 </file>
@@ -1078,7 +1120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AF3F25-4127-44F5-ACE1-35E82582D3CE}">
-  <dimension ref="A4:I57"/>
+  <dimension ref="A4:I65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
@@ -1234,7 +1276,7 @@
         <v>185</v>
       </c>
       <c r="E12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1251,7 +1293,7 @@
         <v>171</v>
       </c>
       <c r="E13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1268,7 +1310,7 @@
         <v>172</v>
       </c>
       <c r="E14" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1285,7 +1327,7 @@
         <v>173</v>
       </c>
       <c r="E15" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1513,10 +1555,10 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E32" t="s">
         <v>192</v>
-      </c>
-      <c r="E32" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1530,10 +1572,10 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E33" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1547,10 +1589,10 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E34" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1563,11 +1605,11 @@
       <c r="C35" t="s">
         <v>78</v>
       </c>
-      <c r="D35" t="s">
-        <v>196</v>
+      <c r="D35" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="E35" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1613,11 +1655,11 @@
       <c r="C39" t="s">
         <v>80</v>
       </c>
-      <c r="D39" t="s">
-        <v>204</v>
+      <c r="D39" s="3" t="s">
+        <v>201</v>
       </c>
       <c r="E39" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1630,11 +1672,11 @@
       <c r="C40" t="s">
         <v>81</v>
       </c>
-      <c r="D40" t="s">
-        <v>200</v>
+      <c r="D40" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="E40" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1647,11 +1689,11 @@
       <c r="C41" t="s">
         <v>82</v>
       </c>
-      <c r="D41" t="s">
-        <v>198</v>
+      <c r="D41" s="2" t="s">
+        <v>195</v>
       </c>
       <c r="E41" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1873,6 +1915,82 @@
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
       <c r="E57" s="7"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>70</v>
+      </c>
+      <c r="B60" t="s">
+        <v>209</v>
+      </c>
+      <c r="D60" t="s">
+        <v>208</v>
+      </c>
+      <c r="E60" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>71</v>
+      </c>
+      <c r="B61" t="s">
+        <v>211</v>
+      </c>
+      <c r="D61" t="s">
+        <v>212</v>
+      </c>
+      <c r="E61" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>73</v>
+      </c>
+      <c r="B62" t="s">
+        <v>214</v>
+      </c>
+      <c r="D62" t="s">
+        <v>213</v>
+      </c>
+      <c r="E62" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>131</v>
+      </c>
+      <c r="B63" t="s">
+        <v>216</v>
+      </c>
+      <c r="D63" t="s">
+        <v>217</v>
+      </c>
+      <c r="E63" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>207</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Added Mode and Select functions for Audio. Added Welcome Screen. Added Mode LED Blink IRQ - All works
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1702360-672E-400F-B1F2-7E9E79B50DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F414446-735A-4292-8091-540F5348F5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -668,9 +668,6 @@
     <t>P14</t>
   </si>
   <si>
-    <t>TEST_IRQ</t>
-  </si>
-  <si>
     <t>T11</t>
   </si>
   <si>
@@ -696,6 +693,9 @@
   </si>
   <si>
     <t>MB_RESET</t>
+  </si>
+  <si>
+    <t>TEST_IRQ (Timer 1 IRQ input to interrupt controller)</t>
   </si>
 </sst>
 </file>
@@ -1937,7 +1937,7 @@
         <v>208</v>
       </c>
       <c r="E60" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1945,13 +1945,13 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
+        <v>210</v>
+      </c>
+      <c r="D61" t="s">
         <v>211</v>
       </c>
-      <c r="D61" t="s">
-        <v>212</v>
-      </c>
       <c r="E61" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1959,13 +1959,13 @@
         <v>73</v>
       </c>
       <c r="B62" t="s">
+        <v>213</v>
+      </c>
+      <c r="D62" t="s">
+        <v>212</v>
+      </c>
+      <c r="E62" t="s">
         <v>214</v>
-      </c>
-      <c r="D62" t="s">
-        <v>213</v>
-      </c>
-      <c r="E62" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1973,13 +1973,13 @@
         <v>131</v>
       </c>
       <c r="B63" t="s">
+        <v>215</v>
+      </c>
+      <c r="D63" t="s">
         <v>216</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>217</v>
-      </c>
-      <c r="E63" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added much code for audio playback, updated circular buffers - not working - it is playing jittery garbage
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F414446-735A-4292-8091-540F5348F5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A668FC8-DF9A-46F6-90BD-377425906986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -1170,7 +1170,7 @@
       <c r="C6" t="s">
         <v>91</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>163</v>
       </c>
       <c r="E6" t="s">
@@ -1190,7 +1190,7 @@
       <c r="C7" t="s">
         <v>92</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>167</v>
       </c>
       <c r="E7" t="s">
@@ -1210,7 +1210,7 @@
       <c r="C8" t="s">
         <v>93</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>169</v>
       </c>
       <c r="E8" t="s">
@@ -1233,7 +1233,7 @@
       <c r="C9" t="s">
         <v>94</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E9" t="s">

</xml_diff>

<commit_message>
Added IMR ADC 7476Ax2 Custom IP. Bug fix in transistion from Signal to Audio mode. Stable signal acquistion at 50KHz - not 75KHz
</commit_message>
<xml_diff>
--- a/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
+++ b/PL_Softcore_SA/PinMap_ArtyA7_To_SSA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\PL_Softcore_SA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A668FC8-DF9A-46F6-90BD-377425906986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7303BEFE-5C1C-4419-B28B-4DC8D3D7B216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{D2802923-92BB-439C-8335-E54F07B9031B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="241">
   <si>
     <t>G13</t>
   </si>
@@ -482,9 +482,6 @@
     <t>Debug Port UART TX</t>
   </si>
   <si>
-    <t>TP4</t>
-  </si>
-  <si>
     <t>USD_CSn[0]</t>
   </si>
   <si>
@@ -554,12 +551,6 @@
     <t>SIG_SEL</t>
   </si>
   <si>
-    <t>TP7</t>
-  </si>
-  <si>
-    <t>TP6</t>
-  </si>
-  <si>
     <t>Legend:</t>
   </si>
   <si>
@@ -599,9 +590,6 @@
     <t>ARTY A7 J4 CONNECTOR</t>
   </si>
   <si>
-    <t>TEST_IO_0</t>
-  </si>
-  <si>
     <t>Audio Enable = 1, Disable = 0 (gpio2_io_o_0[6])</t>
   </si>
   <si>
@@ -650,12 +638,6 @@
     <t>IO Expander common SPI MOSI</t>
   </si>
   <si>
-    <t>Timer 1 Test Signal (gpio2_io_o_0[0] =  TIMER_1_OUTPUT)</t>
-  </si>
-  <si>
-    <t>Timer 2 Test Signal (gpio2_io_o_0[1] = TIMER_2_OUTPUT)</t>
-  </si>
-  <si>
     <t>J4.13</t>
   </si>
   <si>
@@ -680,22 +662,103 @@
     <t>R12</t>
   </si>
   <si>
-    <t>ADC_IRQ_DONE</t>
-  </si>
-  <si>
     <t>T14</t>
   </si>
   <si>
     <t>CK_IO5</t>
   </si>
   <si>
-    <t>DISPLAY_CSn - not used - display uses JD1 - J4.1 for CSn</t>
-  </si>
-  <si>
     <t>MB_RESET</t>
   </si>
   <si>
     <t>TEST_IRQ (Timer 1 IRQ input to interrupt controller)</t>
+  </si>
+  <si>
+    <t>ADC_IP_IRQ</t>
+  </si>
+  <si>
+    <t>ADC PRIMARY IRQ</t>
+  </si>
+  <si>
+    <t>CK_IO6</t>
+  </si>
+  <si>
+    <t>CK_IO7</t>
+  </si>
+  <si>
+    <t>T15</t>
+  </si>
+  <si>
+    <t>T16</t>
+  </si>
+  <si>
+    <t>ADC_IP_IRQ: Primary IRQ for ADC IP 7476Ax2</t>
+  </si>
+  <si>
+    <t>ADC_IRQ_N_DONE: N number of conversions done - indirect IRQ for ADC IP 7476Ax2</t>
+  </si>
+  <si>
+    <t>U16</t>
+  </si>
+  <si>
+    <t>CK_IO1</t>
+  </si>
+  <si>
+    <t>V15</t>
+  </si>
+  <si>
+    <t>CK_IO0</t>
+  </si>
+  <si>
+    <t>TEST_IO_1</t>
+  </si>
+  <si>
+    <t>MB_CLK</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[10]</t>
+  </si>
+  <si>
+    <t>TEST_IRQ</t>
+  </si>
+  <si>
+    <t>MicroBlaze Clock</t>
+  </si>
+  <si>
+    <t>MicroBlaze Reset</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[5]</t>
+  </si>
+  <si>
+    <t>UI_CSn - not used for display - display uses JD1 - J4.1 for CSn</t>
+  </si>
+  <si>
+    <t>UI_CSn</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[9]</t>
+  </si>
+  <si>
+    <t>TEST_IO_0 (TP4 on PCB)</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[0]</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[1]</t>
+  </si>
+  <si>
+    <t>Timer 1 Test Signal ] = TIMER_1_OUTPUT) - TP6 ON PCB</t>
+  </si>
+  <si>
+    <t>Timer 2 Test Signal  =  TIMER_2_OUTPUT) - TP7 ON PCB</t>
+  </si>
+  <si>
+    <t>ADC_IRQ_N_DONE</t>
+  </si>
+  <si>
+    <t>gpio2_io_o_0[5]: N number of conversions done - indirect IRQ for ADC IP 7476Ax2</t>
   </si>
 </sst>
 </file>
@@ -1130,7 +1193,7 @@
   <sheetData>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>64</v>
@@ -1145,19 +1208,19 @@
         <v>133</v>
       </c>
       <c r="H4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="H5" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1171,13 +1234,13 @@
         <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E6" t="s">
         <v>163</v>
       </c>
-      <c r="E6" t="s">
-        <v>164</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1191,13 +1254,13 @@
         <v>92</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" t="s">
         <v>167</v>
       </c>
-      <c r="E7" t="s">
-        <v>168</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1211,16 +1274,16 @@
         <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" t="s">
         <v>169</v>
       </c>
-      <c r="E8" t="s">
-        <v>170</v>
-      </c>
       <c r="H8" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1234,10 +1297,10 @@
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E9" t="s">
         <v>165</v>
-      </c>
-      <c r="E9" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1273,10 +1336,10 @@
         <v>95</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1290,10 +1353,10 @@
         <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E13" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1306,11 +1369,11 @@
       <c r="C14" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>172</v>
+      <c r="D14" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="E14" t="s">
-        <v>204</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1323,11 +1386,11 @@
       <c r="C15" t="s">
         <v>98</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>173</v>
+      <c r="D15" s="2" t="s">
+        <v>235</v>
       </c>
       <c r="E15" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1354,7 +1417,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -1372,10 +1435,10 @@
         <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1389,10 +1452,10 @@
         <v>84</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E20" t="s">
         <v>151</v>
-      </c>
-      <c r="E20" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1406,10 +1469,10 @@
         <v>85</v>
       </c>
       <c r="D21" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E21" t="s">
         <v>154</v>
-      </c>
-      <c r="E21" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1423,10 +1486,10 @@
         <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E22" t="s">
         <v>156</v>
-      </c>
-      <c r="E22" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1462,7 +1525,7 @@
         <v>87</v>
       </c>
       <c r="E25" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1476,7 +1539,7 @@
         <v>88</v>
       </c>
       <c r="E26" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1490,10 +1553,10 @@
         <v>89</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1507,10 +1570,10 @@
         <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E28" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1537,7 +1600,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -1555,10 +1618,10 @@
         <v>75</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1572,10 +1635,10 @@
         <v>76</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E33" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1589,10 +1652,10 @@
         <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E34" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1606,10 +1669,10 @@
         <v>78</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E35" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1644,6 +1707,9 @@
       <c r="C38" t="s">
         <v>79</v>
       </c>
+      <c r="E38" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -1656,10 +1722,10 @@
         <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E39" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1673,10 +1739,10 @@
         <v>81</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E40" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1690,10 +1756,10 @@
         <v>82</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E41" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1720,7 +1786,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -1861,11 +1927,11 @@
       <c r="C53" t="s">
         <v>73</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>148</v>
+      <c r="D53" s="2" t="s">
+        <v>233</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>187</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -1909,7 +1975,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
@@ -1920,24 +1986,51 @@
       <c r="A58" t="s">
         <v>66</v>
       </c>
+      <c r="B58" t="s">
+        <v>222</v>
+      </c>
+      <c r="C58" t="s">
+        <v>223</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E58" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
+      <c r="B59" t="s">
+        <v>220</v>
+      </c>
+      <c r="C59" t="s">
+        <v>221</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E59" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>209</v>
-      </c>
-      <c r="D60" t="s">
-        <v>208</v>
+        <v>203</v>
+      </c>
+      <c r="C60" t="s">
+        <v>202</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>227</v>
       </c>
       <c r="E60" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1945,13 +2038,16 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
+        <v>204</v>
+      </c>
+      <c r="C61" t="s">
+        <v>205</v>
+      </c>
+      <c r="D61" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="D61" t="s">
-        <v>211</v>
-      </c>
       <c r="E61" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1959,13 +2055,16 @@
         <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>213</v>
-      </c>
-      <c r="D62" t="s">
-        <v>212</v>
+        <v>207</v>
+      </c>
+      <c r="C62" t="s">
+        <v>206</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>239</v>
       </c>
       <c r="E62" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1973,23 +2072,50 @@
         <v>131</v>
       </c>
       <c r="B63" t="s">
-        <v>215</v>
-      </c>
-      <c r="D63" t="s">
-        <v>216</v>
+        <v>208</v>
+      </c>
+      <c r="C63" t="s">
+        <v>209</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>232</v>
       </c>
       <c r="E63" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="B64" t="s">
+        <v>216</v>
+      </c>
+      <c r="C64" t="s">
+        <v>214</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E64" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>207</v>
+        <v>201</v>
+      </c>
+      <c r="B65" t="s">
+        <v>217</v>
+      </c>
+      <c r="C65" t="s">
+        <v>215</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E65" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>